<commit_message>
fix: extract sold dates from tx_date on Midland API and rebuild web portal
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-皇廷汇.xlsx
+++ b/files/九龙-九龙塘-皇廷汇.xlsx
@@ -750,7 +750,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2024-03-21</t>
         </is>
       </c>
       <c r="H4" s="5" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2023-08-17</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
@@ -990,7 +990,7 @@
         <is>
           <t>A号屋
 10718呎 (4+房)
-(已售)
+(24年-03月)
 $3.40亿
 $31,722/呎</t>
         </is>
@@ -999,7 +999,7 @@
         <is>
           <t>B号屋
 5845呎 (4+房)
-(已售)
+(23年-08月)
 $2.55亿
 $43,593/呎</t>
         </is>

</xml_diff>